<commit_message>
sms and template validation testcases updated
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_sender_id.xlsx
+++ b/tests/test_data/valid_sender_id.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AUTOTEST1</t>
+          <t>AUTOT1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ENT001</t>
+          <t>1701158046444780002</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,12 +463,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AUTOTEST2</t>
+          <t>AUTOT2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ENT001</t>
+          <t>1701158046444780002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>

<commit_message>
sms failed test update
</commit_message>
<xml_diff>
--- a/tests/test_data/valid_sender_id.xlsx
+++ b/tests/test_data/valid_sender_id.xlsx
@@ -419,22 +419,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Sender ID</t>
+          <t>Sender_ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Entity ID</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Country Code</t>
+          <t>Country_Code</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Entity_ID</t>
         </is>
       </c>
     </row>
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1701158046444780002</t>
+          <t>Transactional</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Auto test sender 1</t>
+          <t>'1701158046444780002'</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1701158046444780002</t>
+          <t>OTP</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,7 +478,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Auto test sender 2</t>
+          <t>'1701158046444780002'</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENT002</t>
+          <t>Promotional</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -498,11 +498,7 @@
           <t>SG</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Auto test sender 3</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -512,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENT002</t>
+          <t>Transactional</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -520,11 +516,7 @@
           <t>SG</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Auto test sender 4</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -534,7 +526,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENT003</t>
+          <t>OTP</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -542,11 +534,7 @@
           <t>MY</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Auto test sender 5</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>